<commit_message>
correct DIC Lab2 codes and results
</commit_message>
<xml_diff>
--- a/DIC/Lab2/Task2/task2.xlsx
+++ b/DIC/Lab2/Task2/task2.xlsx
@@ -446,7 +446,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>f3</t>
+          <t>f4</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -532,54 +532,50 @@
       <c r="B2" t="n">
         <v>4</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>16.0000</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>64.0000</t>
-        </is>
+      <c r="C2" t="n">
+        <v>16</v>
+      </c>
+      <c r="D2" t="n">
+        <v>64</v>
       </c>
       <c r="E2" t="n">
-        <v>8.760000000000001e-12</v>
+        <v>9.125000000000001e-12</v>
       </c>
       <c r="F2" t="n">
-        <v>7.959e-12</v>
+        <v>8.113e-12</v>
       </c>
       <c r="G2" t="n">
-        <v>8.360000000000001e-12</v>
+        <v>8.619e-12</v>
       </c>
       <c r="H2" t="n">
-        <v>2.01e-11</v>
+        <v>6.987e-12</v>
       </c>
       <c r="I2" t="n">
-        <v>1.762e-11</v>
+        <v>6.585e-12</v>
       </c>
       <c r="J2" t="n">
-        <v>1.886e-11</v>
+        <v>6.786e-12</v>
       </c>
       <c r="K2" t="n">
-        <v>6.522e-12</v>
+        <v>6.93e-12</v>
       </c>
       <c r="L2" t="n">
-        <v>5.46e-12</v>
+        <v>6.573e-12</v>
       </c>
       <c r="M2" t="n">
-        <v>5.991e-12</v>
+        <v>6.752e-12</v>
       </c>
       <c r="N2" t="n">
-        <v>8.421000000000001e-12</v>
+        <v>7.279000000000001e-12</v>
       </c>
       <c r="O2" t="n">
-        <v>7.054e-12</v>
+        <v>6.74e-12</v>
       </c>
       <c r="P2" t="n">
-        <v>7.738e-12</v>
+        <v>7.009e-12</v>
       </c>
       <c r="Q2" t="n">
-        <v>4.095e-11</v>
+        <v>2.917e-11</v>
       </c>
       <c r="R2" t="n">
         <v>25</v>
@@ -595,54 +591,50 @@
       <c r="B3" t="n">
         <v>4</v>
       </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>15.0000</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>60.0000</t>
-        </is>
+      <c r="C3" t="n">
+        <v>15</v>
+      </c>
+      <c r="D3" t="n">
+        <v>60</v>
       </c>
       <c r="E3" t="n">
-        <v>8.752e-12</v>
+        <v>9.114e-12</v>
       </c>
       <c r="F3" t="n">
-        <v>7.837000000000001e-12</v>
+        <v>8.1e-12</v>
       </c>
       <c r="G3" t="n">
-        <v>8.295000000000001e-12</v>
+        <v>8.607e-12</v>
       </c>
       <c r="H3" t="n">
-        <v>1.898e-11</v>
+        <v>6.741e-12</v>
       </c>
       <c r="I3" t="n">
-        <v>1.654e-11</v>
+        <v>6.355e-12</v>
       </c>
       <c r="J3" t="n">
-        <v>1.776e-11</v>
+        <v>6.548e-12</v>
       </c>
       <c r="K3" t="n">
-        <v>6.531e-12</v>
+        <v>6.828e-12</v>
       </c>
       <c r="L3" t="n">
-        <v>5.494e-12</v>
+        <v>6.459e-12</v>
       </c>
       <c r="M3" t="n">
-        <v>6.012e-12</v>
+        <v>6.644e-12</v>
       </c>
       <c r="N3" t="n">
-        <v>8.342e-12</v>
+        <v>7.556000000000001e-12</v>
       </c>
       <c r="O3" t="n">
-        <v>7.227e-12</v>
+        <v>6.985e-12</v>
       </c>
       <c r="P3" t="n">
-        <v>7.785e-12</v>
+        <v>7.271e-12</v>
       </c>
       <c r="Q3" t="n">
-        <v>3.986e-11</v>
+        <v>2.907e-11</v>
       </c>
       <c r="R3" t="n">
         <v>25</v>
@@ -658,54 +650,50 @@
       <c r="B4" t="n">
         <v>4</v>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>20.0000</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>80.0000</t>
-        </is>
+      <c r="C4" t="n">
+        <v>20</v>
+      </c>
+      <c r="D4" t="n">
+        <v>80</v>
       </c>
       <c r="E4" t="n">
-        <v>8.740999999999999e-12</v>
+        <v>9.102999999999999e-12</v>
       </c>
       <c r="F4" t="n">
-        <v>8.116e-12</v>
+        <v>8.1e-12</v>
       </c>
       <c r="G4" t="n">
-        <v>8.427999999999999e-12</v>
+        <v>8.602000000000001e-12</v>
       </c>
       <c r="H4" t="n">
-        <v>2.427e-11</v>
+        <v>7.975e-12</v>
       </c>
       <c r="I4" t="n">
-        <v>2.103e-11</v>
+        <v>7.503e-12</v>
       </c>
       <c r="J4" t="n">
-        <v>2.265e-11</v>
+        <v>7.739e-12</v>
       </c>
       <c r="K4" t="n">
-        <v>7.162e-12</v>
+        <v>7.365e-12</v>
       </c>
       <c r="L4" t="n">
-        <v>5.696e-12</v>
+        <v>7.01e-12</v>
       </c>
       <c r="M4" t="n">
-        <v>6.429e-12</v>
+        <v>7.188e-12</v>
       </c>
       <c r="N4" t="n">
-        <v>8.647000000000001e-12</v>
+        <v>6.468e-12</v>
       </c>
       <c r="O4" t="n">
-        <v>7.211e-12</v>
+        <v>5.995e-12</v>
       </c>
       <c r="P4" t="n">
-        <v>7.929e-12</v>
+        <v>6.232e-12</v>
       </c>
       <c r="Q4" t="n">
-        <v>4.543e-11</v>
+        <v>2.976e-11</v>
       </c>
       <c r="R4" t="n">
         <v>25</v>
@@ -721,54 +709,50 @@
       <c r="B5" t="n">
         <v>5</v>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>16.0000</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>64.0000</t>
-        </is>
+      <c r="C5" t="n">
+        <v>16</v>
+      </c>
+      <c r="D5" t="n">
+        <v>64</v>
       </c>
       <c r="E5" t="n">
-        <v>9.935000000000001e-12</v>
+        <v>1.03e-11</v>
       </c>
       <c r="F5" t="n">
-        <v>8.942e-12</v>
+        <v>9.197e-12</v>
       </c>
       <c r="G5" t="n">
-        <v>9.439e-12</v>
+        <v>9.749e-12</v>
       </c>
       <c r="H5" t="n">
-        <v>1.678e-11</v>
+        <v>6.463e-12</v>
       </c>
       <c r="I5" t="n">
-        <v>1.499e-11</v>
+        <v>6.096e-12</v>
       </c>
       <c r="J5" t="n">
-        <v>1.588e-11</v>
+        <v>6.279e-12</v>
       </c>
       <c r="K5" t="n">
-        <v>6.043e-12</v>
+        <v>6.685e-12</v>
       </c>
       <c r="L5" t="n">
-        <v>5.158e-12</v>
+        <v>6.269e-12</v>
       </c>
       <c r="M5" t="n">
-        <v>5.6e-12</v>
+        <v>6.477e-12</v>
       </c>
       <c r="N5" t="n">
-        <v>7.837000000000001e-12</v>
+        <v>7.217e-12</v>
       </c>
       <c r="O5" t="n">
-        <v>6.674e-12</v>
+        <v>6.7e-12</v>
       </c>
       <c r="P5" t="n">
-        <v>7.255e-12</v>
+        <v>6.958e-12</v>
       </c>
       <c r="Q5" t="n">
-        <v>3.818e-11</v>
+        <v>2.946e-11</v>
       </c>
       <c r="R5" t="n">
         <v>25</v>
@@ -784,54 +768,50 @@
       <c r="B6" t="n">
         <v>5</v>
       </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>15.0000</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>60.0000</t>
-        </is>
+      <c r="C6" t="n">
+        <v>15</v>
+      </c>
+      <c r="D6" t="n">
+        <v>60</v>
       </c>
       <c r="E6" t="n">
-        <v>1.003e-11</v>
+        <v>1.029e-11</v>
       </c>
       <c r="F6" t="n">
-        <v>8.956e-12</v>
+        <v>9.218000000000001e-12</v>
       </c>
       <c r="G6" t="n">
-        <v>9.492e-12</v>
+        <v>9.753e-12</v>
       </c>
       <c r="H6" t="n">
-        <v>1.589e-11</v>
+        <v>6.248e-12</v>
       </c>
       <c r="I6" t="n">
-        <v>1.428e-11</v>
+        <v>5.893e-12</v>
       </c>
       <c r="J6" t="n">
-        <v>1.509e-11</v>
+        <v>6.071e-12</v>
       </c>
       <c r="K6" t="n">
-        <v>5.821e-12</v>
+        <v>6.595e-12</v>
       </c>
       <c r="L6" t="n">
-        <v>5.19e-12</v>
+        <v>6.175e-12</v>
       </c>
       <c r="M6" t="n">
-        <v>5.506e-12</v>
+        <v>6.385e-12</v>
       </c>
       <c r="N6" t="n">
-        <v>7.630999999999999e-12</v>
+        <v>7.504e-12</v>
       </c>
       <c r="O6" t="n">
-        <v>6.846e-12</v>
+        <v>6.952e-12</v>
       </c>
       <c r="P6" t="n">
-        <v>7.238e-12</v>
+        <v>7.228e-12</v>
       </c>
       <c r="Q6" t="n">
-        <v>3.732e-11</v>
+        <v>2.944e-11</v>
       </c>
       <c r="R6" t="n">
         <v>25</v>
@@ -847,54 +827,50 @@
       <c r="B7" t="n">
         <v>5</v>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>20.0000</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>80.0000</t>
-        </is>
+      <c r="C7" t="n">
+        <v>20</v>
+      </c>
+      <c r="D7" t="n">
+        <v>80</v>
       </c>
       <c r="E7" t="n">
-        <v>9.895e-12</v>
+        <v>1.025e-11</v>
       </c>
       <c r="F7" t="n">
-        <v>8.932e-12</v>
+        <v>9.197e-12</v>
       </c>
       <c r="G7" t="n">
-        <v>9.414e-12</v>
+        <v>9.723e-12</v>
       </c>
       <c r="H7" t="n">
-        <v>2.042e-11</v>
+        <v>7.283e-12</v>
       </c>
       <c r="I7" t="n">
-        <v>1.789e-11</v>
+        <v>6.889e-12</v>
       </c>
       <c r="J7" t="n">
-        <v>1.916e-11</v>
+        <v>7.086e-12</v>
       </c>
       <c r="K7" t="n">
-        <v>6.435e-12</v>
+        <v>7.045e-12</v>
       </c>
       <c r="L7" t="n">
-        <v>5.09e-12</v>
+        <v>6.637e-12</v>
       </c>
       <c r="M7" t="n">
-        <v>5.762e-12</v>
+        <v>6.841e-12</v>
       </c>
       <c r="N7" t="n">
-        <v>8.273000000000001e-12</v>
+        <v>6.385e-12</v>
       </c>
       <c r="O7" t="n">
-        <v>6.619e-12</v>
+        <v>5.948e-12</v>
       </c>
       <c r="P7" t="n">
-        <v>7.446e-12</v>
+        <v>6.166e-12</v>
       </c>
       <c r="Q7" t="n">
-        <v>4.178e-11</v>
+        <v>2.982e-11</v>
       </c>
       <c r="R7" t="n">
         <v>25</v>

</xml_diff>